<commit_message>
Artigo finalizado: auditoria completa, SIM real, RAIS 2018-2025, RPPS, slides Rmd, README com tabela de fontes
</commit_message>
<xml_diff>
--- a/dados/manifesto/manifesto_arquivos.xlsx
+++ b/dados/manifesto/manifesto_arquivos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P85"/>
+  <dimension ref="A1:P128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5379,49 +5379,33 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/abastecimento_agua_censo_2022.csv</t>
+          <t>dados/brutos/cnes-rh/cnes_rh_campos_201812_controle.prn</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>abastecimento_agua_censo_2022.csv</t>
+          <t>cnes_rh_campos_201812_controle.prn</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.prn</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>8324</t>
+          <t>94</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2026-07-18T10:52:16</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>utf-8</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>,</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>66</t>
-        </is>
-      </c>
+          <t>2026-07-18T12:49:42</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -5430,68 +5414,48 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>2b7e08d88986044d6f009f343e0aa6daf9a96a806dc14c2af6ab01b226a6444e</t>
+          <t>4c0d1b879fc06b37bf06d7276535bb3f82fa5645a38466d7f6c8db9d14ca3b95</t>
         </is>
       </c>
       <c r="M67" t="inlineStr"/>
       <c r="N67" t="inlineStr"/>
       <c r="O67" t="inlineStr">
         <is>
-          <t>bruto (fonte IBGE/SIDRA)</t>
-        </is>
-      </c>
-      <c r="P67" t="inlineStr">
-        <is>
-          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
-        </is>
-      </c>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/estimativas_populacionais.csv</t>
+          <t>dados/brutos/cnes-rh/cnes_rh_campos_201812_ocupacoes.prn</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>estimativas_populacionais.csv</t>
+          <t>cnes_rh_campos_201812_ocupacoes.prn</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.prn</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2511</t>
+          <t>9163</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>2026-07-18T10:52:16</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>utf-8</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>,</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
+          <t>2026-07-18T12:49:42</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
       <c r="J68" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -5500,68 +5464,48 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>5afc076b1e5dc706c67e638f55e886abdd9ce936df7d91c9e5351256b7131963</t>
+          <t>ac05fc95dd76b127cf8ba9bdaa3d2f15a4d891f952267eb3fe31c96952553f08</t>
         </is>
       </c>
       <c r="M68" t="inlineStr"/>
       <c r="N68" t="inlineStr"/>
       <c r="O68" t="inlineStr">
         <is>
-          <t>bruto (fonte IBGE/SIDRA)</t>
-        </is>
-      </c>
-      <c r="P68" t="inlineStr">
-        <is>
-          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
-        </is>
-      </c>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/extracao_vegetal_silvicultura.csv</t>
+          <t>dados/brutos/cnes-rh/cnes_rh_campos_201912_controle.prn</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>extracao_vegetal_silvicultura.csv</t>
+          <t>cnes_rh_campos_201912_controle.prn</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.prn</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>623186</t>
+          <t>96</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>2026-07-18T10:52:16</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>utf-8</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>,</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>4212</t>
-        </is>
-      </c>
+          <t>2026-07-18T12:49:45</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
       <c r="J69" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -5570,68 +5514,48 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>850916e770700dc47a550d276cd79ef2d6ed8e3e370db412eb225a1652598e2a</t>
+          <t>c38fc35fd9fd6ca97199e9dfbceace4ecbd26a843fb59b99658cf081c165e9bb</t>
         </is>
       </c>
       <c r="M69" t="inlineStr"/>
       <c r="N69" t="inlineStr"/>
       <c r="O69" t="inlineStr">
         <is>
-          <t>bruto (fonte IBGE/SIDRA)</t>
-        </is>
-      </c>
-      <c r="P69" t="inlineStr">
-        <is>
-          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
-        </is>
-      </c>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/instrucao_censo_2022.csv</t>
+          <t>dados/brutos/cnes-rh/cnes_rh_campos_201912_ocupacoes.prn</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>instrucao_censo_2022.csv</t>
+          <t>cnes_rh_campos_201912_ocupacoes.prn</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.prn</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>186970</t>
+          <t>9362</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2026-07-18T10:52:16</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>utf-8</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>,</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>1080</t>
-        </is>
-      </c>
+          <t>2026-07-18T12:49:45</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -5640,68 +5564,48 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>f0188a358c2f27e8bb556d6d8045c2582b55bad440554818564150ba17a7d746</t>
+          <t>cb7eae4eeba23c58c7da44649b02831a9f3769f3c368282d6073702cc11158c2</t>
         </is>
       </c>
       <c r="M70" t="inlineStr"/>
       <c r="N70" t="inlineStr"/>
       <c r="O70" t="inlineStr">
         <is>
-          <t>bruto (fonte IBGE/SIDRA)</t>
-        </is>
-      </c>
-      <c r="P70" t="inlineStr">
-        <is>
-          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
-        </is>
-      </c>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/log_download_sidra.csv</t>
+          <t>dados/brutos/cnes-rh/cnes_rh_campos_202012_controle.prn</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>log_download_sidra.csv</t>
+          <t>cnes_rh_campos_202012_controle.prn</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.prn</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>1456</t>
+          <t>96</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2026-07-18T10:52:16</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>utf-8</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>,</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
+          <t>2026-07-18T12:49:47</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -5710,68 +5614,48 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>d65519852238bbc7edcaab243c7f0e81bba614f3bad3df3b33e44d2f36e6c71e</t>
+          <t>fef47a416db03d7ec1fa3044a5e35a50a62f6905cf461fdc2a054a1a0dd8eacf</t>
         </is>
       </c>
       <c r="M71" t="inlineStr"/>
       <c r="N71" t="inlineStr"/>
       <c r="O71" t="inlineStr">
         <is>
-          <t>bruto (fonte IBGE/SIDRA)</t>
-        </is>
-      </c>
-      <c r="P71" t="inlineStr">
-        <is>
-          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
-        </is>
-      </c>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/pecuaria_municipal_rebanhos.csv</t>
+          <t>dados/brutos/cnes-rh/cnes_rh_campos_202012_ocupacoes.prn</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>pecuaria_municipal_rebanhos.csv</t>
+          <t>cnes_rh_campos_202012_ocupacoes.prn</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.prn</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>60721</t>
+          <t>9380</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>2026-07-18T10:52:16</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>utf-8</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>,</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>510</t>
-        </is>
-      </c>
+          <t>2026-07-18T12:49:47</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -5780,68 +5664,48 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>22994a871228f36b3ecca31cddc245cdc4827ab16b582e3e42210f53124021c7</t>
+          <t>cdde48725cf7a901956d7d0d935f58cb50b47e6231836b044073642317fb93c1</t>
         </is>
       </c>
       <c r="M72" t="inlineStr"/>
       <c r="N72" t="inlineStr"/>
       <c r="O72" t="inlineStr">
         <is>
-          <t>bruto (fonte IBGE/SIDRA)</t>
-        </is>
-      </c>
-      <c r="P72" t="inlineStr">
-        <is>
-          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
-        </is>
-      </c>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/pib_municipal.csv</t>
+          <t>dados/brutos/cnes-rh/cnes_rh_campos_202112_controle.prn</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>pib_municipal.csv</t>
+          <t>cnes_rh_campos_202112_controle.prn</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.prn</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>254111</t>
+          <t>96</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2026-07-18T10:52:16</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>utf-8</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>,</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>1012</t>
-        </is>
-      </c>
+          <t>2026-07-18T12:49:50</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -5850,68 +5714,48 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>7b40e39980c1988723d07ff43230d5ad95a4877599b6cc2f751829a4475310c1</t>
+          <t>9a7f9a865eebd07e5a0c3aedd2904e15357a67047b6e839ed75b8d5888edd727</t>
         </is>
       </c>
       <c r="M73" t="inlineStr"/>
       <c r="N73" t="inlineStr"/>
       <c r="O73" t="inlineStr">
         <is>
-          <t>bruto (fonte IBGE/SIDRA)</t>
-        </is>
-      </c>
-      <c r="P73" t="inlineStr">
-        <is>
-          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
-        </is>
-      </c>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/pib_per_capita.csv</t>
+          <t>dados/brutos/cnes-rh/cnes_rh_campos_202112_ocupacoes.prn</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>pib_per_capita.csv</t>
+          <t>cnes_rh_campos_202112_ocupacoes.prn</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.prn</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>511</t>
+          <t>9350</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>2026-07-18T10:52:16</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>utf-8</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>,</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+          <t>2026-07-18T12:49:50</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
       <c r="J74" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -5920,68 +5764,48 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>9b051cae6c9b3e7ad3e584bea62fd9a48dd11384a6ee1b9bccdbbbe035043290</t>
+          <t>c1a9433110bc66afba0244e3674f85c1c44ec646fb662f841344bbc7968496b7</t>
         </is>
       </c>
       <c r="M74" t="inlineStr"/>
       <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr">
         <is>
-          <t>bruto (fonte IBGE/SIDRA)</t>
-        </is>
-      </c>
-      <c r="P74" t="inlineStr">
-        <is>
-          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
-        </is>
-      </c>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/populacao_area_densidade_censo_2022.csv</t>
+          <t>dados/brutos/cnes-rh/cnes_rh_campos_202212_controle.prn</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>populacao_area_densidade_censo_2022.csv</t>
+          <t>cnes_rh_campos_202212_controle.prn</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.prn</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>517</t>
+          <t>96</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>2026-07-18T10:52:16</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>utf-8</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>,</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+          <t>2026-07-18T12:49:53</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -5990,68 +5814,48 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>698f5ac06f8895efbf0ee5828bdd4ea7ff266ef34694d389c2dc6688c7a2b22a</t>
+          <t>be035256cfff6dbdd26d6f598b11b8fa75c1f85b1ba63a99b7611ade1d9ce34f</t>
         </is>
       </c>
       <c r="M75" t="inlineStr"/>
       <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr">
         <is>
-          <t>bruto (fonte IBGE/SIDRA)</t>
-        </is>
-      </c>
-      <c r="P75" t="inlineStr">
-        <is>
-          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
-        </is>
-      </c>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/populacao_cor_raca_censo_2022.csv</t>
+          <t>dados/brutos/cnes-rh/cnes_rh_campos_202212_ocupacoes.prn</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>populacao_cor_raca_censo_2022.csv</t>
+          <t>cnes_rh_campos_202212_ocupacoes.prn</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.prn</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>324684</t>
+          <t>9289</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2026-07-18T10:52:16</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>utf-8</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>,</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>2412</t>
-        </is>
-      </c>
+          <t>2026-07-18T12:49:53</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -6060,68 +5864,48 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>e2aac8250bf6929855b09a7b1b26d473a4da205a602033a94d59860d519c371c</t>
+          <t>c1b50a71d56552ce485a226775920bcaad81007ec7f1d6f3cf39638f44135da7</t>
         </is>
       </c>
       <c r="M76" t="inlineStr"/>
       <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr">
         <is>
-          <t>bruto (fonte IBGE/SIDRA)</t>
-        </is>
-      </c>
-      <c r="P76" t="inlineStr">
-        <is>
-          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
-        </is>
-      </c>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/populacao_por_sexo_idade_2022.csv</t>
+          <t>dados/brutos/cnes-rh/cnes_rh_campos_202312_controle.prn</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>populacao_por_sexo_idade_2022.csv</t>
+          <t>cnes_rh_campos_202312_controle.prn</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.prn</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>171961</t>
+          <t>96</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>2026-07-18T10:52:16</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>utf-8</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>,</t>
-        </is>
-      </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>1206</t>
-        </is>
-      </c>
+          <t>2026-07-18T12:49:56</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -6130,68 +5914,48 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>e1335944983b43cf652a8430670842d9fbcbd7018e95c56db06c23b9661e9446</t>
+          <t>d59421800ede66c705e71a05caceec7832448d8f2ffda60716204b77b2259b93</t>
         </is>
       </c>
       <c r="M77" t="inlineStr"/>
       <c r="N77" t="inlineStr"/>
       <c r="O77" t="inlineStr">
         <is>
-          <t>bruto (fonte IBGE/SIDRA)</t>
-        </is>
-      </c>
-      <c r="P77" t="inlineStr">
-        <is>
-          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
-        </is>
-      </c>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/populacao_residente_censo_2022.csv</t>
+          <t>dados/brutos/cnes-rh/cnes_rh_campos_202312_ocupacoes.prn</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>populacao_residente_censo_2022.csv</t>
+          <t>cnes_rh_campos_202312_ocupacoes.prn</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.prn</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>863</t>
+          <t>9462</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>2026-07-18T10:52:16</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>utf-8</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>,</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
+          <t>2026-07-18T12:49:56</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -6200,68 +5964,48 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>ea7bb2d875b0d8ee78c6c14d63a3c2cd1515e8e3f7df27251d9673b0a1235126</t>
+          <t>39d849014be6d12aa453cd4ea44e2357d829253da70df3e852632cc3a413772b</t>
         </is>
       </c>
       <c r="M78" t="inlineStr"/>
       <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr">
         <is>
-          <t>bruto (fonte IBGE/SIDRA)</t>
-        </is>
-      </c>
-      <c r="P78" t="inlineStr">
-        <is>
-          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
-        </is>
-      </c>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/producao_agricola_lavoura_permanente.csv</t>
+          <t>dados/brutos/cnes-rh/cnes_rh_campos_202412_controle.prn</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>producao_agricola_lavoura_permanente.csv</t>
+          <t>cnes_rh_campos_202412_controle.prn</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.prn</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>1236616</t>
+          <t>96</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>2026-07-18T10:52:16</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>utf-8</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>,</t>
-        </is>
-      </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>9945</t>
-        </is>
-      </c>
+          <t>2026-07-18T12:49:59</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -6270,68 +6014,48 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>05f117e295b9e74e12abc5c877f985f2be9f212885e4e075ac4218eaaa2f4223</t>
+          <t>81d70c99d84469231e71fc1199442da73c6351bcae9db62c70208103c0f5b51e</t>
         </is>
       </c>
       <c r="M79" t="inlineStr"/>
       <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr">
         <is>
-          <t>bruto (fonte IBGE/SIDRA)</t>
-        </is>
-      </c>
-      <c r="P79" t="inlineStr">
-        <is>
-          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
-        </is>
-      </c>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/producao_agricola_lavoura_temporaria.csv</t>
+          <t>dados/brutos/cnes-rh/cnes_rh_campos_202412_ocupacoes.prn</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>producao_agricola_lavoura_temporaria.csv</t>
+          <t>cnes_rh_campos_202412_ocupacoes.prn</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.prn</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>1060359</t>
+          <t>9476</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2026-07-18T10:52:16</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>utf-8</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>,</t>
-        </is>
-      </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>8670</t>
-        </is>
-      </c>
+          <t>2026-07-18T12:49:59</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
       <c r="J80" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -6340,68 +6064,48 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>f3fdb6e6112e97d0174402dbe4e0b5e7d9b19b2e543cb7506168d18de3f53dc2</t>
+          <t>91e3fa734da03c3585e08fd50f36739a4d91ebc4c879e40c5e0fbcf07a14cb69</t>
         </is>
       </c>
       <c r="M80" t="inlineStr"/>
       <c r="N80" t="inlineStr"/>
       <c r="O80" t="inlineStr">
         <is>
-          <t>bruto (fonte IBGE/SIDRA)</t>
-        </is>
-      </c>
-      <c r="P80" t="inlineStr">
-        <is>
-          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
-        </is>
-      </c>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/producao_origem_animal.csv</t>
+          <t>dados/brutos/cnes-rh/cnes_rh_campos_202512_controle.prn</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>producao_origem_animal.csv</t>
+          <t>cnes_rh_campos_202512_controle.prn</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.prn</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>86993</t>
+          <t>96</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>2026-07-18T10:52:16</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>utf-8</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>,</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>714</t>
-        </is>
-      </c>
+          <t>2026-07-18T12:50:02</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
       <c r="J81" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -6410,68 +6114,48 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>cac2f50d943583ca8377e481f47d1c8d8c891d08623f3dbb33ee8845194ff728</t>
+          <t>f5adebbe24f9e5c55f66e61737c85d45d9985fdcc52c8d8ac84fc59a71a9b0f6</t>
         </is>
       </c>
       <c r="M81" t="inlineStr"/>
       <c r="N81" t="inlineStr"/>
       <c r="O81" t="inlineStr">
         <is>
-          <t>bruto (fonte IBGE/SIDRA)</t>
-        </is>
-      </c>
-      <c r="P81" t="inlineStr">
-        <is>
-          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
-        </is>
-      </c>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>referencias/CBO2002_Ocupacao_cartaproale.csv</t>
+          <t>dados/brutos/cnes-rh/cnes_rh_campos_202512_ocupacoes.prn</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>CBO2002_Ocupacao_cartaproale.csv</t>
+          <t>cnes_rh_campos_202512_ocupacoes.prn</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.prn</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>109417</t>
+          <t>10116</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>2026-07-18T11:35:01</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>latin-1</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>;</t>
-        </is>
-      </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>2719</t>
-        </is>
-      </c>
+          <t>2026-07-18T12:50:02</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -6480,14 +6164,14 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>a374b4061c8986b29ec7677fbdb33175917108d27984a60e700f40539c4d32ca</t>
+          <t>a23838c5709a6027fdb080a99dbdecb314d19e3b41950160eb391edbaff8f899</t>
         </is>
       </c>
       <c r="M82" t="inlineStr"/>
       <c r="N82" t="inlineStr"/>
       <c r="O82" t="inlineStr">
         <is>
-          <t>tabela de validação CBO (espelho público)</t>
+          <t>intermediário/derivado legado</t>
         </is>
       </c>
       <c r="P82" t="inlineStr"/>
@@ -6495,33 +6179,49 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>referencias/dicionario-cat-dados-abertos-10-02-2021.xlsx</t>
+          <t>dados/brutos/ibge/Cadastro Central de Empresas - Campos dos Goytacazes.csv</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>dicionario-cat-dados-abertos-10-02-2021.xlsx</t>
+          <t>Cadastro Central de Empresas - Campos dos Goytacazes.csv</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>.xlsx</t>
+          <t>.csv</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>10405</t>
+          <t>6715</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>2026-07-18T10:51:47</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr"/>
-      <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
+          <t>2026-07-18T20:03:18</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>;</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>115</t>
+        </is>
+      </c>
       <c r="J83" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -6530,14 +6230,14 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>5405d1af10d3e764a08bc8a319f836348dca346bc14eddf380e6235fdba26b84</t>
+          <t>389d2d19dc290df74646c194a999741c36147554fd82223477e8b3600af5a25e</t>
         </is>
       </c>
       <c r="M83" t="inlineStr"/>
       <c r="N83" t="inlineStr"/>
       <c r="O83" t="inlineStr">
         <is>
-          <t>documentação da fonte (INSS)</t>
+          <t>intermediário/derivado legado</t>
         </is>
       </c>
       <c r="P83" t="inlineStr"/>
@@ -6545,33 +6245,49 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>referencias/fonte_cbo.txt</t>
+          <t>dados/brutos/ibge/Finanças públicas - Campos dos Goytacazes.csv</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>fonte_cbo.txt</t>
+          <t>Finanças públicas - Campos dos Goytacazes.csv</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>.txt</t>
+          <t>.csv</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>583</t>
+          <t>4847</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2026-07-18T11:50:09</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr"/>
+          <t>2026-07-18T20:03:42</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>;</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="J84" t="inlineStr">
         <is>
           <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
@@ -6580,7 +6296,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>10a27bd97ff2283674fd7b15ad3139ae72ecfe9040a0464f8b8dd78a1c098725</t>
+          <t>b9971e225c9768f42b1b3b01eef62e6cd7b58f5c703ecd65fd41999534a6ed52</t>
         </is>
       </c>
       <c r="M84" t="inlineStr"/>
@@ -6595,27 +6311,27 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>referencias/tabela_referencias_abnt.xlsx</t>
+          <t>dados/brutos/rais/RAIS_2018_MG_ES_RJ.7z.part</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>tabela_referencias_abnt.xlsx</t>
+          <t>RAIS_2018_MG_ES_RJ.7z.part</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>.xlsx</t>
+          <t>.part</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>6579</t>
+          <t>554485187</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2026-07-18T11:50:09</t>
+          <t>2026-07-18T19:04:27</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -6630,7 +6346,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>5845645ff04d14e1e53df1eea63507e1c873fb6416dc9f3ef063fcc47f050745</t>
+          <t>ead23e232693d13ef6b1a907fb7213e73d6d0b605770a7807d9c583afd5bd098</t>
         </is>
       </c>
       <c r="M85" t="inlineStr"/>
@@ -6641,6 +6357,2572 @@
         </is>
       </c>
       <c r="P85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>dados/brutos/rais/RAIS_2018_MG_ES_RJ_test</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>RAIS_2018_MG_ES_RJ_test</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>2026-07-18T17:15:11</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>e3b0c44298fc1c149afbf4c8996fb92427ae41e4649b934ca495991b7852b855</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr"/>
+      <c r="N86" t="inlineStr"/>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>dados/brutos/rais/RAIS_2019_MG_ES_RJ.7z.part</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>RAIS_2019_MG_ES_RJ.7z.part</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>.part</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>101354656</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>2026-07-18T19:07:33</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>bb5c916af801fbb15cca890ba69f7f792e23f28884db08a17ab84ba155db2710</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>dados/brutos/rais/RAIS_2019_MG_ES_RJ_test</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>RAIS_2019_MG_ES_RJ_test</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>2026-07-18T17:26:24</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>e3b0c44298fc1c149afbf4c8996fb92427ae41e4649b934ca495991b7852b855</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr"/>
+      <c r="N88" t="inlineStr"/>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>dados/brutos/rais/RAIS_2020_MG_ES_RJ.7z.part</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>RAIS_2020_MG_ES_RJ.7z.part</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>.part</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>33423360</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>2026-07-18T19:09:43</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>a5517297b99ceeae6011aaf28221fa5c22a119ee3c896f5d8d6bee10c34783e1</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr"/>
+      <c r="N89" t="inlineStr"/>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>dados/brutos/rais/RAIS_2020_MG_ES_RJ_test</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>RAIS_2020_MG_ES_RJ_test</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>2026-07-18T17:37:40</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>e3b0c44298fc1c149afbf4c8996fb92427ae41e4649b934ca495991b7852b855</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr"/>
+      <c r="N90" t="inlineStr"/>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>dados/brutos/rais/RAIS_2021_MG_ES_RJ.7z.part</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>RAIS_2021_MG_ES_RJ.7z.part</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>.part</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>104460080</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>2026-07-18T19:19:22</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>f9867c7caa58dee82a41755ed3a297e70b3dcd59c95657251da99cce1e11d534</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr"/>
+      <c r="N91" t="inlineStr"/>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>dados/brutos/rais/RAIS_2021_MG_ES_RJ_test</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>RAIS_2021_MG_ES_RJ_test</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>2026-07-18T17:48:24</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>e3b0c44298fc1c149afbf4c8996fb92427ae41e4649b934ca495991b7852b855</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr"/>
+      <c r="N92" t="inlineStr"/>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>dados/brutos/rais/RAIS_2022_MG_ES_RJ_test</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>RAIS_2022_MG_ES_RJ_test</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>2026-07-18T18:02:13</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>e3b0c44298fc1c149afbf4c8996fb92427ae41e4649b934ca495991b7852b855</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>dados/brutos/rais/RAIS_2023_MG_ES_RJ.7z</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>RAIS_2023_MG_ES_RJ.7z</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>.7z</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>715072048</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>2026-07-18T17:05:58</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>159827a4172adb81ecc9e40d25a55222bf4a1946d1e245fafe265a2ba9fbbc88</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr"/>
+      <c r="N94" t="inlineStr"/>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>dados/brutos/rais/RAIS_2024_MG_ES_RJ.7z.part</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>RAIS_2024_MG_ES_RJ.7z.part</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>.part</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>747149815</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>2026-07-18T19:30:56</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>15d59d8eab7766875a75daf2ba657f072811b3805a5d23371f19bb2f814207cc</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr"/>
+      <c r="N95" t="inlineStr"/>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>dados/brutos/rais/RAIS_2024_MG_ES_RJ_test</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>RAIS_2024_MG_ES_RJ_test</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>2026-07-18T18:14:54</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>e3b0c44298fc1c149afbf4c8996fb92427ae41e4649b934ca495991b7852b855</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr"/>
+      <c r="N96" t="inlineStr"/>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>dados/brutos/rais/RAIS_2025_MG_ES_RJ.7z</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>RAIS_2025_MG_ES_RJ.7z</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>.7z</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>766814132</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>2026-07-18T18:32:43</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>d9c4e359fa16c6a1f929f49c8aec0201a9fbfb801964dc2e27032914924f1f15</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr"/>
+      <c r="N97" t="inlineStr"/>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>dados/brutos/rais/RAIS_2025_MG_ES_RJ_test</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>RAIS_2025_MG_ES_RJ_test</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr"/>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>2026-07-18T18:32:43</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>e3b0c44298fc1c149afbf4c8996fb92427ae41e4649b934ca495991b7852b855</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr"/>
+      <c r="N98" t="inlineStr"/>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>dados/brutos/sidra-campos/abastecimento_agua_censo_2022.csv</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>abastecimento_agua_censo_2022.csv</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>8324</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>2026-07-18T10:52:16</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>2b7e08d88986044d6f009f343e0aa6daf9a96a806dc14c2af6ab01b226a6444e</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr"/>
+      <c r="N99" t="inlineStr"/>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>bruto (fonte IBGE/SIDRA)</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>dados/brutos/sidra-campos/estimativas_populacionais.csv</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>estimativas_populacionais.csv</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>2511</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>2026-07-18T10:52:16</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>5afc076b1e5dc706c67e638f55e886abdd9ce936df7d91c9e5351256b7131963</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr"/>
+      <c r="N100" t="inlineStr"/>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>bruto (fonte IBGE/SIDRA)</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>dados/brutos/sidra-campos/extracao_vegetal_silvicultura.csv</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>extracao_vegetal_silvicultura.csv</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>623186</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>2026-07-18T10:52:16</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>4212</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>850916e770700dc47a550d276cd79ef2d6ed8e3e370db412eb225a1652598e2a</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr"/>
+      <c r="N101" t="inlineStr"/>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>bruto (fonte IBGE/SIDRA)</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>dados/brutos/sidra-campos/instrucao_censo_2022.csv</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>instrucao_censo_2022.csv</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>186970</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>2026-07-18T10:52:16</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>1080</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>f0188a358c2f27e8bb556d6d8045c2582b55bad440554818564150ba17a7d746</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr"/>
+      <c r="N102" t="inlineStr"/>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>bruto (fonte IBGE/SIDRA)</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>dados/brutos/sidra-campos/log_download_sidra.csv</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>log_download_sidra.csv</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>1456</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>2026-07-18T10:52:16</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>d65519852238bbc7edcaab243c7f0e81bba614f3bad3df3b33e44d2f36e6c71e</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr"/>
+      <c r="N103" t="inlineStr"/>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>bruto (fonte IBGE/SIDRA)</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>dados/brutos/sidra-campos/pecuaria_municipal_rebanhos.csv</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>pecuaria_municipal_rebanhos.csv</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>60721</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>2026-07-18T10:52:16</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>510</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>22994a871228f36b3ecca31cddc245cdc4827ab16b582e3e42210f53124021c7</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr"/>
+      <c r="N104" t="inlineStr"/>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>bruto (fonte IBGE/SIDRA)</t>
+        </is>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>dados/brutos/sidra-campos/pib_municipal.csv</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>pib_municipal.csv</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>254111</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>2026-07-18T10:52:16</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>1012</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>7b40e39980c1988723d07ff43230d5ad95a4877599b6cc2f751829a4475310c1</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr"/>
+      <c r="N105" t="inlineStr"/>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>bruto (fonte IBGE/SIDRA)</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>dados/brutos/sidra-campos/populacao_area_densidade_censo_2022.csv</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>populacao_area_densidade_censo_2022.csv</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>517</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>2026-07-18T10:52:16</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>698f5ac06f8895efbf0ee5828bdd4ea7ff266ef34694d389c2dc6688c7a2b22a</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr"/>
+      <c r="N106" t="inlineStr"/>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>bruto (fonte IBGE/SIDRA)</t>
+        </is>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>dados/brutos/sidra-campos/populacao_cor_raca_censo_2022.csv</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>populacao_cor_raca_censo_2022.csv</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>324684</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>2026-07-18T10:52:16</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>2412</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>e2aac8250bf6929855b09a7b1b26d473a4da205a602033a94d59860d519c371c</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr"/>
+      <c r="N107" t="inlineStr"/>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>bruto (fonte IBGE/SIDRA)</t>
+        </is>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>dados/brutos/sidra-campos/populacao_por_sexo_idade_2022.csv</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>populacao_por_sexo_idade_2022.csv</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>171961</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>2026-07-18T10:52:16</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>1206</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>e1335944983b43cf652a8430670842d9fbcbd7018e95c56db06c23b9661e9446</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr"/>
+      <c r="N108" t="inlineStr"/>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>bruto (fonte IBGE/SIDRA)</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>dados/brutos/sidra-campos/populacao_residente_censo_2022.csv</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>populacao_residente_censo_2022.csv</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>863</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>2026-07-18T10:52:16</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>ea7bb2d875b0d8ee78c6c14d63a3c2cd1515e8e3f7df27251d9673b0a1235126</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr"/>
+      <c r="N109" t="inlineStr"/>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>bruto (fonte IBGE/SIDRA)</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>dados/brutos/sidra-campos/populacao_residente_taxa_crescimento.csv</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>populacao_residente_taxa_crescimento.csv</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>511</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>2026-07-18T10:52:16</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>9b051cae6c9b3e7ad3e584bea62fd9a48dd11384a6ee1b9bccdbbbe035043290</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr"/>
+      <c r="N110" t="inlineStr"/>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>bruto (fonte IBGE/SIDRA)</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>dados/brutos/sidra-campos/producao_agricola_lavoura_permanente.csv</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>producao_agricola_lavoura_permanente.csv</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>1236616</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>2026-07-18T10:52:16</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>9945</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr"/>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>05f117e295b9e74e12abc5c877f985f2be9f212885e4e075ac4218eaaa2f4223</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr"/>
+      <c r="N111" t="inlineStr"/>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>bruto (fonte IBGE/SIDRA)</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>dados/brutos/sidra-campos/producao_agricola_lavoura_temporaria.csv</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>producao_agricola_lavoura_temporaria.csv</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>1060359</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>2026-07-18T10:52:16</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>8670</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr"/>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>f3fdb6e6112e97d0174402dbe4e0b5e7d9b19b2e543cb7506168d18de3f53dc2</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr"/>
+      <c r="N112" t="inlineStr"/>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>bruto (fonte IBGE/SIDRA)</t>
+        </is>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>dados/brutos/sidra-campos/producao_origem_animal.csv</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>producao_origem_animal.csv</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>86993</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>2026-07-18T10:52:16</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>714</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr"/>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>cac2f50d943583ca8377e481f47d1c8d8c891d08623f3dbb33ee8845194ff728</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr"/>
+      <c r="N113" t="inlineStr"/>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>bruto (fonte IBGE/SIDRA)</t>
+        </is>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>legado: scripts/legado/CARACTERIZACAO_script_original.R</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>dados/brutos/sim/DORJ2023.dbc</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>DORJ2023.dbc</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>.dbc</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>11382859</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:11:08</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr"/>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>c988dd824c5c1be7cb7d6266fb828c289a4806b069feaed1c84133069fa20d07</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr"/>
+      <c r="N114" t="inlineStr"/>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>dados/brutos/sim/DORJ2023.dbf</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>DORJ2023.dbf</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>.dbf</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>2818</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:19:32</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr"/>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>5f4d123a1b10b49432351e0fced21d3c5f9610a3f70f3747a1e808476d0c6bb7</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr"/>
+      <c r="N115" t="inlineStr"/>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>dados/brutos/sim/DORJ2023_v2.dbf</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>DORJ2023_v2.dbf</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>.dbf</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>2818</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:18:43</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr"/>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>52854181c7dd817b537bd7478784483cb115e6eb8aa9d251498dc06dad480ee3</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr"/>
+      <c r="N116" t="inlineStr"/>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>dados/brutos/sim/SIM_Campos_2019.csv</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>SIM_Campos_2019.csv</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>1857625</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:30:54</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>4299</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr"/>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>8d3b8045329c3b7d13b5b31542a78a58e16d66a14339829b6103d102e897caa6</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr"/>
+      <c r="N117" t="inlineStr"/>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>dados/brutos/sim/SIM_Campos_2020.csv</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>SIM_Campos_2020.csv</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>2084332</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:31:04</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>4831</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr"/>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>76c4419da1504716081521c8e663365c36cdb3abd3c615165aacf61e7045b845</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr"/>
+      <c r="N118" t="inlineStr"/>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>dados/brutos/sim/SIM_Campos_2021.csv</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>SIM_Campos_2021.csv</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>2457292</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:31:12</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>5635</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>b2b9892322c7ed342545889c10e0c2cd2cf83204c5dfdac0389ec833db1d7166</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr"/>
+      <c r="N119" t="inlineStr"/>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>dados/brutos/sim/SIM_Campos_2022.csv</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>SIM_Campos_2022.csv</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>1988794</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:31:19</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>4608</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr"/>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>47a83a0842a604483b2d43026ef07952258871a6a6e7e0dae7c6128fee96bead</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr"/>
+      <c r="N120" t="inlineStr"/>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>dados/brutos/sim/SIM_Campos_2023.csv</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>SIM_Campos_2023.csv</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>1810840</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:31:26</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>4199</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr"/>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>f9add46c2cc74adea458876ca7029febdb7a382943ac2e57345e37ba27c70451</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr"/>
+      <c r="N121" t="inlineStr"/>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>dados/brutos/sim/SIM_Campos_2024.csv</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>SIM_Campos_2024.csv</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>1870051</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:31:32</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>4346</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>54a91249ccfcafa8cfd57b9b283dc0f71cee5fc5cb08ac5766298353aa4b31e6</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr"/>
+      <c r="N122" t="inlineStr"/>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>dados/brutos/sim/SIM_Campos_mortalidade.csv</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>SIM_Campos_mortalidade.csv</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:24:11</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>latin-1</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>;</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr"/>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>21a57d2939ec7a2df472c4cfaae78a776062ea3abb2ff87fd7dec76490839c9d</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr"/>
+      <c r="N123" t="inlineStr"/>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>referencias/CBO2002_Ocupacao_cartaproale.csv</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>CBO2002_Ocupacao_cartaproale.csv</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>109417</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>2026-07-18T11:35:01</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>latin-1</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>;</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>2719</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr"/>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>a374b4061c8986b29ec7677fbdb33175917108d27984a60e700f40539c4d32ca</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr"/>
+      <c r="N124" t="inlineStr"/>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>tabela de validação CBO (espelho público)</t>
+        </is>
+      </c>
+      <c r="P124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>referencias/dicionario-cat-dados-abertos-10-02-2021.xlsx</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>dicionario-cat-dados-abertos-10-02-2021.xlsx</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>.xlsx</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>10405</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>2026-07-18T10:51:47</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>5405d1af10d3e764a08bc8a319f836348dca346bc14eddf380e6235fdba26b84</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr"/>
+      <c r="N125" t="inlineStr"/>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>documentação da fonte (INSS)</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>referencias/fonte_cbo.txt</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>fonte_cbo.txt</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>.txt</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>583</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>2026-07-18T13:36:18</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr"/>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>10a27bd97ff2283674fd7b15ad3139ae72ecfe9040a0464f8b8dd78a1c098725</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr"/>
+      <c r="N126" t="inlineStr"/>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>referencias/tabela_referencias_abnt.xlsx</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>tabela_referencias_abnt.xlsx</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>.xlsx</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>6570</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>2026-07-18T13:36:18</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>efe0bbdd5b62aa4795eedfd15ed9c8aea22320551c8ff3a73ff4782be3a889de</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr"/>
+      <c r="N127" t="inlineStr"/>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>referencias/tabela_referencias_abnt_atualizada.csv</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>tabela_referencias_abnt_atualizada.csv</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>2221</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>2026-07-18T13:36:10</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>utf-8-sig</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>;</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>NAO — nenhum arquivo SmartLab presente (etapa excluída por decisão metodológica)</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr"/>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>ed096c7ef71fc12dfe17926d7524013b14356ffe6a8ea1065b13e8080b79af8d</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr"/>
+      <c r="N128" t="inlineStr"/>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>intermediário/derivado legado</t>
+        </is>
+      </c>
+      <c r="P128" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: CI requirements, gitignore CAGED .7z, CSVs regenerados
</commit_message>
<xml_diff>
--- a/dados/manifesto/manifesto_arquivos.xlsx
+++ b/dados/manifesto/manifesto_arquivos.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,82 +429,82 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>caminho_relativo</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>nome</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>extensao</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>tamanho_bytes</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>modificado_em</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>codificacao</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>separador</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>n_colunas</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>n_linhas_dados</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>smartlab</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>problema_leitura</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>sha256</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>esquema</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>linhas_malformadas</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>condicao</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>scripts_associados</t>
         </is>
@@ -801,7 +813,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202101.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202101.csv</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -879,7 +891,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202104.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202104.csv</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -957,7 +969,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202107.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202107.csv</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1035,7 +1047,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202110.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202110.csv</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1113,7 +1125,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202201.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202201.csv</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1191,7 +1203,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202204.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202204.csv</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1269,7 +1281,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202207.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202207.csv</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1347,7 +1359,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202208.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202208.csv</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1425,7 +1437,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202209.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202209.csv</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1503,7 +1515,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202210.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202210.csv</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1581,7 +1593,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202211.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202211.csv</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1659,7 +1671,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202212.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202212.csv</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1737,7 +1749,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202301.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202301.csv</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1815,7 +1827,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202302.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202302.csv</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1893,7 +1905,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202303.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202303.csv</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1971,7 +1983,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202304.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202304.csv</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2049,7 +2061,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202305.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202305.csv</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2127,7 +2139,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202306.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202306.csv</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2205,7 +2217,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202307.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202307.csv</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2283,7 +2295,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202308.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202308.csv</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2361,7 +2373,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202309.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202309.csv</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2439,7 +2451,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202310.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202310.csv</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2517,7 +2529,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202311.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202311.csv</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2595,7 +2607,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202312.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202312.csv</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2673,7 +2685,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202401.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202401.csv</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2751,7 +2763,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202402.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202402.csv</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2829,7 +2841,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202403.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202403.csv</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2907,7 +2919,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202404.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202404.csv</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2985,7 +2997,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202405.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202405.csv</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3063,7 +3075,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202406.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202406.csv</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3141,7 +3153,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202407.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202407.csv</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3219,7 +3231,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202408.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202408.csv</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3297,7 +3309,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202409.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202409.csv</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3375,7 +3387,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202410.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202410.csv</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3453,7 +3465,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202411.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202411.csv</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3531,7 +3543,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202412.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202412.csv</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3609,7 +3621,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202501.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202501.csv</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3687,7 +3699,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202502.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202502.csv</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3765,7 +3777,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202503.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202503.csv</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3843,7 +3855,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202504.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202504.csv</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3921,7 +3933,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202505.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202505.csv</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3999,7 +4011,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202506.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202506.csv</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -4077,7 +4089,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202507.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202507.csv</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -4155,7 +4167,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202508.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202508.csv</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -4233,7 +4245,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202509.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202509.csv</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -4311,7 +4323,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202510.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202510.csv</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -4389,7 +4401,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202511.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202511.csv</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -4467,7 +4479,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/D.SDA.PDA.005.CAT.202512.csv</t>
+          <t>banco de dados/cat-inss/D.SDA.PDA.005.CAT.202512.csv</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -4545,7 +4557,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/README.md</t>
+          <t>banco de dados/cat-inss/README.md</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -4599,7 +4611,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/cat-comp-outnovdez-2018.csv</t>
+          <t>banco de dados/cat-inss/cat-comp-outnovdez-2018.csv</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -4677,7 +4689,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/cat-comp01-02-03-2020.csv</t>
+          <t>banco de dados/cat-inss/cat-comp01-02-03-2020.csv</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -4755,7 +4767,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/cat-comp04-05-06-2019.csv</t>
+          <t>banco de dados/cat-inss/cat-comp04-05-06-2019.csv</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -4833,7 +4845,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/cat-comp07-08-09-2019.csv</t>
+          <t>banco de dados/cat-inss/cat-comp07-08-09-2019.csv</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -4911,7 +4923,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/cat-comp10-11-12-2019.csv</t>
+          <t>banco de dados/cat-inss/cat-comp10-11-12-2019.csv</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -4989,7 +5001,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/cat-comp10-11-12-2020.csv</t>
+          <t>banco de dados/cat-inss/cat-comp10-11-12-2020.csv</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -5067,7 +5079,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/cat-competencia-04-05-06-2020.csv</t>
+          <t>banco de dados/cat-inss/cat-competencia-04-05-06-2020.csv</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -5145,7 +5157,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/cat-competencia-07-08-09-2020.csv</t>
+          <t>banco de dados/cat-inss/cat-competencia-07-08-09-2020.csv</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -5223,7 +5235,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/cat-jul-ago-set-2018.csv</t>
+          <t>banco de dados/cat-inss/cat-jul-ago-set-2018.csv</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -5301,7 +5313,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>dados/brutos/cat-inss/cat2018-comp01-02-03-2019.csv</t>
+          <t>banco de dados/cat-inss/cat2018-comp01-02-03-2019.csv</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -5379,7 +5391,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>dados/brutos/cnes-rh/cnes_rh_campos_201812_controle.prn</t>
+          <t>banco de dados/cnes/cnes_rh_campos_201812_controle.prn</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -5429,7 +5441,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>dados/brutos/cnes-rh/cnes_rh_campos_201812_ocupacoes.prn</t>
+          <t>banco de dados/cnes/cnes_rh_campos_201812_ocupacoes.prn</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -5479,7 +5491,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>dados/brutos/cnes-rh/cnes_rh_campos_201912_controle.prn</t>
+          <t>banco de dados/cnes/cnes_rh_campos_201912_controle.prn</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -5529,7 +5541,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>dados/brutos/cnes-rh/cnes_rh_campos_201912_ocupacoes.prn</t>
+          <t>banco de dados/cnes/cnes_rh_campos_201912_ocupacoes.prn</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -5579,7 +5591,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>dados/brutos/cnes-rh/cnes_rh_campos_202012_controle.prn</t>
+          <t>banco de dados/cnes/cnes_rh_campos_202012_controle.prn</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -5629,7 +5641,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>dados/brutos/cnes-rh/cnes_rh_campos_202012_ocupacoes.prn</t>
+          <t>banco de dados/cnes/cnes_rh_campos_202012_ocupacoes.prn</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -5679,7 +5691,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>dados/brutos/cnes-rh/cnes_rh_campos_202112_controle.prn</t>
+          <t>banco de dados/cnes/cnes_rh_campos_202112_controle.prn</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -5729,7 +5741,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>dados/brutos/cnes-rh/cnes_rh_campos_202112_ocupacoes.prn</t>
+          <t>banco de dados/cnes/cnes_rh_campos_202112_ocupacoes.prn</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -5779,7 +5791,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>dados/brutos/cnes-rh/cnes_rh_campos_202212_controle.prn</t>
+          <t>banco de dados/cnes/cnes_rh_campos_202212_controle.prn</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -5829,7 +5841,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>dados/brutos/cnes-rh/cnes_rh_campos_202212_ocupacoes.prn</t>
+          <t>banco de dados/cnes/cnes_rh_campos_202212_ocupacoes.prn</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -5879,7 +5891,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>dados/brutos/cnes-rh/cnes_rh_campos_202312_controle.prn</t>
+          <t>banco de dados/cnes/cnes_rh_campos_202312_controle.prn</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -5929,7 +5941,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>dados/brutos/cnes-rh/cnes_rh_campos_202312_ocupacoes.prn</t>
+          <t>banco de dados/cnes/cnes_rh_campos_202312_ocupacoes.prn</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -5979,7 +5991,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>dados/brutos/cnes-rh/cnes_rh_campos_202412_controle.prn</t>
+          <t>banco de dados/cnes/cnes_rh_campos_202412_controle.prn</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -6029,7 +6041,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>dados/brutos/cnes-rh/cnes_rh_campos_202412_ocupacoes.prn</t>
+          <t>banco de dados/cnes/cnes_rh_campos_202412_ocupacoes.prn</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -6079,7 +6091,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>dados/brutos/cnes-rh/cnes_rh_campos_202512_controle.prn</t>
+          <t>banco de dados/cnes/cnes_rh_campos_202512_controle.prn</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -6129,7 +6141,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>dados/brutos/cnes-rh/cnes_rh_campos_202512_ocupacoes.prn</t>
+          <t>banco de dados/cnes/cnes_rh_campos_202512_ocupacoes.prn</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -6179,7 +6191,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>dados/brutos/ibge/Cadastro Central de Empresas - Campos dos Goytacazes.csv</t>
+          <t>banco de dados/ibge/Cadastro Central de Empresas - Campos dos Goytacazes.csv</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -6245,7 +6257,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>dados/brutos/ibge/Finanças públicas - Campos dos Goytacazes.csv</t>
+          <t>banco de dados/ibge/Finanças públicas - Campos dos Goytacazes.csv</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -6311,7 +6323,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>dados/brutos/rais/RAIS_2018_MG_ES_RJ.7z.part</t>
+          <t>banco de dados/rais/RAIS_2018_MG_ES_RJ.7z.part</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -6361,7 +6373,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>dados/brutos/rais/RAIS_2018_MG_ES_RJ_test</t>
+          <t>banco de dados/rais/RAIS_2018_MG_ES_RJ_test</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -6407,7 +6419,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>dados/brutos/rais/RAIS_2019_MG_ES_RJ.7z.part</t>
+          <t>banco de dados/rais/RAIS_2019_MG_ES_RJ.7z.part</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -6457,7 +6469,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>dados/brutos/rais/RAIS_2019_MG_ES_RJ_test</t>
+          <t>banco de dados/rais/RAIS_2019_MG_ES_RJ_test</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -6503,7 +6515,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>dados/brutos/rais/RAIS_2020_MG_ES_RJ.7z.part</t>
+          <t>banco de dados/rais/RAIS_2020_MG_ES_RJ.7z.part</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -6553,7 +6565,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>dados/brutos/rais/RAIS_2020_MG_ES_RJ_test</t>
+          <t>banco de dados/rais/RAIS_2020_MG_ES_RJ_test</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -6599,7 +6611,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>dados/brutos/rais/RAIS_2021_MG_ES_RJ.7z.part</t>
+          <t>banco de dados/rais/RAIS_2021_MG_ES_RJ.7z.part</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -6649,7 +6661,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>dados/brutos/rais/RAIS_2021_MG_ES_RJ_test</t>
+          <t>banco de dados/rais/RAIS_2021_MG_ES_RJ_test</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -6695,7 +6707,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>dados/brutos/rais/RAIS_2022_MG_ES_RJ_test</t>
+          <t>banco de dados/rais/RAIS_2022_MG_ES_RJ_test</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -6741,7 +6753,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>dados/brutos/rais/RAIS_2023_MG_ES_RJ.7z</t>
+          <t>banco de dados/rais/RAIS_2023_MG_ES_RJ.7z</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -6791,7 +6803,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>dados/brutos/rais/RAIS_2024_MG_ES_RJ.7z.part</t>
+          <t>banco de dados/rais/RAIS_2024_MG_ES_RJ.7z.part</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -6841,7 +6853,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>dados/brutos/rais/RAIS_2024_MG_ES_RJ_test</t>
+          <t>banco de dados/rais/RAIS_2024_MG_ES_RJ_test</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -6887,7 +6899,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>dados/brutos/rais/RAIS_2025_MG_ES_RJ.7z</t>
+          <t>banco de dados/rais/RAIS_2025_MG_ES_RJ.7z</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -6937,7 +6949,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>dados/brutos/rais/RAIS_2025_MG_ES_RJ_test</t>
+          <t>banco de dados/rais/RAIS_2025_MG_ES_RJ_test</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -6983,7 +6995,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/abastecimento_agua_censo_2022.csv</t>
+          <t>banco de dados/sidra-campos/abastecimento_agua_censo_2022.csv</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -7053,7 +7065,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/estimativas_populacionais.csv</t>
+          <t>banco de dados/sidra-campos/estimativas_populacionais.csv</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -7123,7 +7135,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/extracao_vegetal_silvicultura.csv</t>
+          <t>banco de dados/sidra-campos/extracao_vegetal_silvicultura.csv</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -7193,7 +7205,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/instrucao_censo_2022.csv</t>
+          <t>banco de dados/sidra-campos/instrucao_censo_2022.csv</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -7263,7 +7275,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/log_download_sidra.csv</t>
+          <t>banco de dados/sidra-campos/log_download_sidra.csv</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -7333,7 +7345,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/pecuaria_municipal_rebanhos.csv</t>
+          <t>banco de dados/sidra-campos/pecuaria_municipal_rebanhos.csv</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -7403,7 +7415,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/pib_municipal.csv</t>
+          <t>banco de dados/sidra-campos/pib_municipal.csv</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -7473,7 +7485,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/populacao_area_densidade_censo_2022.csv</t>
+          <t>banco de dados/sidra-campos/populacao_area_densidade_censo_2022.csv</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -7543,7 +7555,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/populacao_cor_raca_censo_2022.csv</t>
+          <t>banco de dados/sidra-campos/populacao_cor_raca_censo_2022.csv</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -7613,7 +7625,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/populacao_por_sexo_idade_2022.csv</t>
+          <t>banco de dados/sidra-campos/populacao_por_sexo_idade_2022.csv</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -7683,7 +7695,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/populacao_residente_censo_2022.csv</t>
+          <t>banco de dados/sidra-campos/populacao_residente_censo_2022.csv</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -7753,7 +7765,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/populacao_residente_taxa_crescimento.csv</t>
+          <t>banco de dados/sidra-campos/populacao_residente_taxa_crescimento.csv</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -7823,7 +7835,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/producao_agricola_lavoura_permanente.csv</t>
+          <t>banco de dados/sidra-campos/producao_agricola_lavoura_permanente.csv</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -7893,7 +7905,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/producao_agricola_lavoura_temporaria.csv</t>
+          <t>banco de dados/sidra-campos/producao_agricola_lavoura_temporaria.csv</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -7963,7 +7975,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>dados/brutos/sidra-campos/producao_origem_animal.csv</t>
+          <t>banco de dados/sidra-campos/producao_origem_animal.csv</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -8033,7 +8045,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>dados/brutos/sim/DORJ2023.dbc</t>
+          <t>banco de dados/sim/DORJ2023.dbc</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -8083,7 +8095,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>dados/brutos/sim/DORJ2023.dbf</t>
+          <t>banco de dados/sim/DORJ2023.dbf</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -8133,7 +8145,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>dados/brutos/sim/DORJ2023_v2.dbf</t>
+          <t>banco de dados/sim/DORJ2023_v2.dbf</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -8183,7 +8195,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>dados/brutos/sim/SIM_Campos_2019.csv</t>
+          <t>banco de dados/sim/SIM_Campos_2019.csv</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -8249,7 +8261,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>dados/brutos/sim/SIM_Campos_2020.csv</t>
+          <t>banco de dados/sim/SIM_Campos_2020.csv</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -8315,7 +8327,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>dados/brutos/sim/SIM_Campos_2021.csv</t>
+          <t>banco de dados/sim/SIM_Campos_2021.csv</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -8381,7 +8393,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>dados/brutos/sim/SIM_Campos_2022.csv</t>
+          <t>banco de dados/sim/SIM_Campos_2022.csv</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -8447,7 +8459,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>dados/brutos/sim/SIM_Campos_2023.csv</t>
+          <t>banco de dados/sim/SIM_Campos_2023.csv</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -8513,7 +8525,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>dados/brutos/sim/SIM_Campos_2024.csv</t>
+          <t>banco de dados/sim/SIM_Campos_2024.csv</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -8579,7 +8591,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>dados/brutos/sim/SIM_Campos_mortalidade.csv</t>
+          <t>banco de dados/sim/SIM_Campos_mortalidade.csv</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">

</xml_diff>